<commit_message>
feat: added download excel
</commit_message>
<xml_diff>
--- a/src/assets/plantillas/plantilla.xlsx
+++ b/src/assets/plantillas/plantilla.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F40DF2A0-0ACF-42BD-8069-AA4245937457}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1890" yWindow="3630" windowWidth="18780" windowHeight="13470" xr2:uid="{988331E5-A366-E643-8FED-460F5DF3471D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{988331E5-A366-E643-8FED-460F5DF3471D}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -181,7 +181,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -202,7 +202,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -570,7 +569,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:8" s="10" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>7</v>
       </c>

</xml_diff>